<commit_message>
Cleaned files and added an ignore list
</commit_message>
<xml_diff>
--- a/Marksheet.xlsx
+++ b/Marksheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Saiedur Rahaman Documents\Teaching\COIT12209 Data Science\2025 T1\Assignments - 2025 T1\Assignment 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cqu365-my.sharepoint.com/personal/lachlan_wyer_cqumail_com/Documents/2026/COIT12209/Assignment 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491BDBF9-07FD-48D9-B2A0-AD146DA7472B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{491BDBF9-07FD-48D9-B2A0-AD146DA7472B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31350CE6-799D-4ACA-A31D-1470E3716E32}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19543" windowHeight="12377" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -649,6 +649,33 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -681,33 +708,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -990,51 +990,51 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:L28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="15.7265625" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" customWidth="1"/>
-    <col min="5" max="5" width="19.1796875" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" customWidth="1"/>
-    <col min="7" max="8" width="16.1796875" customWidth="1"/>
-    <col min="9" max="9" width="31.453125" customWidth="1"/>
-    <col min="11" max="11" width="15.54296875" customWidth="1"/>
-    <col min="12" max="12" width="24.26953125" customWidth="1"/>
+    <col min="2" max="2" width="15.61328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.4609375" customWidth="1"/>
+    <col min="4" max="4" width="20.4609375" customWidth="1"/>
+    <col min="5" max="5" width="19.15234375" customWidth="1"/>
+    <col min="6" max="6" width="19.23046875" customWidth="1"/>
+    <col min="7" max="8" width="16.15234375" customWidth="1"/>
+    <col min="9" max="9" width="31.4609375" customWidth="1"/>
+    <col min="11" max="11" width="15.53515625" customWidth="1"/>
+    <col min="12" max="12" width="24.23046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B1" s="50" t="s">
+    <row r="1" spans="2:12" ht="21" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="B1" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="52"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="61"/>
       <c r="E1" s="39"/>
       <c r="F1" s="39"/>
     </row>
-    <row r="2" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="45"/>
-    </row>
-    <row r="3" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C2" s="53"/>
+      <c r="D2" s="54"/>
+    </row>
+    <row r="3" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B3" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="47"/>
-    </row>
-    <row r="4" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="55"/>
+      <c r="D3" s="56"/>
+    </row>
+    <row r="4" spans="2:12" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="48"/>
-      <c r="D4" s="49"/>
-    </row>
-    <row r="5" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:12" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="C4" s="57"/>
+      <c r="D4" s="58"/>
+    </row>
+    <row r="5" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="6" spans="2:12" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="13" t="s">
         <v>17</v>
       </c>
@@ -1063,7 +1063,7 @@
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
     </row>
-    <row r="7" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B7" s="14" t="s">
         <v>6</v>
       </c>
@@ -1081,9 +1081,9 @@
       <c r="H7" s="22">
         <v>0</v>
       </c>
-      <c r="I7" s="42"/>
-    </row>
-    <row r="8" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I7" s="51"/>
+    </row>
+    <row r="8" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B8" s="14" t="s">
         <v>7</v>
       </c>
@@ -1101,9 +1101,9 @@
       <c r="H8" s="6">
         <v>0</v>
       </c>
-      <c r="I8" s="42"/>
-    </row>
-    <row r="9" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I8" s="51"/>
+    </row>
+    <row r="9" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B9" s="14" t="s">
         <v>8</v>
       </c>
@@ -1121,9 +1121,9 @@
       <c r="H9" s="22">
         <v>0</v>
       </c>
-      <c r="I9" s="42"/>
-    </row>
-    <row r="10" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I9" s="51"/>
+    </row>
+    <row r="10" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B10" s="14" t="s">
         <v>9</v>
       </c>
@@ -1139,9 +1139,9 @@
         <v>3</v>
       </c>
       <c r="H10" s="10"/>
-      <c r="I10" s="42"/>
-    </row>
-    <row r="11" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I10" s="51"/>
+    </row>
+    <row r="11" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B11" s="14" t="s">
         <v>10</v>
       </c>
@@ -1157,9 +1157,9 @@
         <v>2</v>
       </c>
       <c r="H11" s="16"/>
-      <c r="I11" s="42"/>
-    </row>
-    <row r="12" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I11" s="51"/>
+    </row>
+    <row r="12" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B12" s="14" t="s">
         <v>11</v>
       </c>
@@ -1175,9 +1175,9 @@
         <v>2</v>
       </c>
       <c r="H12" s="10"/>
-      <c r="I12" s="42"/>
-    </row>
-    <row r="13" spans="2:12" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I12" s="51"/>
+    </row>
+    <row r="13" spans="2:12" s="1" customFormat="1" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B13" s="14" t="s">
         <v>12</v>
       </c>
@@ -1193,9 +1193,9 @@
         <v>3</v>
       </c>
       <c r="H13" s="16"/>
-      <c r="I13" s="42"/>
-    </row>
-    <row r="14" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I13" s="51"/>
+    </row>
+    <row r="14" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B14" s="14" t="s">
         <v>13</v>
       </c>
@@ -1211,9 +1211,9 @@
         <v>2</v>
       </c>
       <c r="H14" s="10"/>
-      <c r="I14" s="42"/>
-    </row>
-    <row r="15" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I14" s="51"/>
+    </row>
+    <row r="15" spans="2:12" ht="15.9" x14ac:dyDescent="0.45">
       <c r="B15" s="14" t="s">
         <v>14</v>
       </c>
@@ -1229,9 +1229,9 @@
         <v>2</v>
       </c>
       <c r="H15" s="16"/>
-      <c r="I15" s="42"/>
-    </row>
-    <row r="16" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="I15" s="51"/>
+    </row>
+    <row r="16" spans="2:12" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B16" s="15" t="s">
         <v>15</v>
       </c>
@@ -1251,12 +1251,12 @@
         <v>4</v>
       </c>
       <c r="H16" s="11"/>
-      <c r="I16" s="43"/>
+      <c r="I16" s="52"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:12" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B17" s="5"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -1269,7 +1269,7 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
     </row>
-    <row r="18" spans="2:12" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:12" ht="32.15" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1287,109 +1287,109 @@
       <c r="K18" s="3"/>
       <c r="L18" s="1"/>
     </row>
-    <row r="19" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B19" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B20" s="53"/>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="55"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B21" s="56"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="58"/>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B22" s="56"/>
-      <c r="C22" s="57"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="58"/>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B23" s="56"/>
-      <c r="C23" s="57"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="58"/>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B24" s="56"/>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="58"/>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B25" s="56"/>
-      <c r="C25" s="57"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="58"/>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B26" s="56"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="58"/>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B27" s="56"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="58"/>
-    </row>
-    <row r="28" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="59"/>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="61"/>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B20" s="42"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="43"/>
+      <c r="I20" s="44"/>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B21" s="45"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="47"/>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B22" s="45"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
+      <c r="I22" s="47"/>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B23" s="45"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="47"/>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B24" s="45"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="47"/>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B25" s="45"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="47"/>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B26" s="45"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="46"/>
+      <c r="I26" s="47"/>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B27" s="45"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="47"/>
+    </row>
+    <row r="28" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B28" s="48"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
+      <c r="I28" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B1:D1"/>
     <mergeCell ref="B20:I28"/>
     <mergeCell ref="I7:I16"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1397,21 +1397,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F9D7ADE019B24D4AAAAA0213A3A82109" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="deb070066159fbb66c8e930a5b8a049d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c11b0a56-fba2-41a9-ac92-e3d69f4d3112" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f0ffcddb8ad961ad72870a1e7e64783" ns3:_="">
     <xsd:import namespace="c11b0a56-fba2-41a9-ac92-e3d69f4d3112"/>
@@ -1543,31 +1528,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E29416F0-7AA8-40D9-9A9F-B107C2D0B8F2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c11b0a56-fba2-41a9-ac92-e3d69f4d3112"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E6F9DEB-CC92-4A7A-A75F-1ECCFEB8C82E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F54FDD88-B560-476F-AA02-696E4B9F8C42}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1585,6 +1561,30 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E6F9DEB-CC92-4A7A-A75F-1ECCFEB8C82E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E29416F0-7AA8-40D9-9A9F-B107C2D0B8F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c11b0a56-fba2-41a9-ac92-e3d69f4d3112"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{a8816c53-b0d3-4c1a-a10e-aa4784cf6e23}" enabled="1" method="Privileged" siteId="{fdade0c4-3fea-4320-ae53-1a1742aeff1e}" contentBits="0" removed="0"/>

</xml_diff>